<commit_message>
docs(m2): importar a entrega m2 tal como extraída do ZIP original
Conteúdo do ZIP submetido para a milestone m2 (cumulativo, inclui m1).
Adiciona os artefactos da m2 e os documentos de reuniões e backlogs do S01/S02.
Ficheiros da m1 que diferem do commit anterior (grelha de rotação m1-v01,
proposta de sistema e declaração de âmbito v01) e templates com bytes
diferentes ficam registados aqui exatamente como estavam no ZIP.
Commit feito a 16/10/2026; não reflete a data original da submissão.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0127oRZG9jPKZ3ii2Fopg1W8
</commit_message>
<xml_diff>
--- a/01-artefactos-de-gestao/01.01-templates/backlog-projeto-template-v05.xlsx
+++ b/01-artefactos-de-gestao/01.01-templates/backlog-projeto-template-v05.xlsx
@@ -5206,13 +5206,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3325336D-D9A3-418C-98EB-E39BD798FB5E}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7855ED32-D8D5-45D4-B0B8-F2C65BAFB002}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{00594BEE-584D-4618-BF92-8D1829A02A8D}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{39D79A0F-63C8-41AD-B4A5-CD901E113A79}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{615ED68D-BF90-4A46-AADE-48E3FD6BE194}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F78A0E2-6DE6-467D-901D-C2D2D14E514B}"/>
 </file>
</xml_diff>

<commit_message>
Migração de dados do Sharepoint
Esta migração de dados pretende uniformizar o local de desenvolvimento no GitHub.
</commit_message>
<xml_diff>
--- a/01-artefactos-de-gestao/01.01-templates/backlog-projeto-template-v05.xlsx
+++ b/01-artefactos-de-gestao/01.01-templates/backlog-projeto-template-v05.xlsx
@@ -5053,9 +5053,10 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100293B981485C9E24DAE651C97D9FBC267" ma:contentTypeVersion="3" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="81e1889baf096e0f1fabc7e628f510b3">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="32f33a6e-f018-4796-a6d6-b8c30f0661e9" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4b8b816b6954550eb9ea5c593f5cc868" ns2:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100293B981485C9E24DAE651C97D9FBC267" ma:contentTypeVersion="9" ma:contentTypeDescription="Criar um novo documento." ma:contentTypeScope="" ma:versionID="67106ac685bde41cc0caab8279921af5">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="32f33a6e-f018-4796-a6d6-b8c30f0661e9" xmlns:ns3="59ec22bb-74c1-4c3c-af96-122e757b18d2" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="6a225e97788944c998cfd0bee463245c" ns2:_="" ns3:_="">
     <xsd:import namespace="32f33a6e-f018-4796-a6d6-b8c30f0661e9"/>
+    <xsd:import namespace="59ec22bb-74c1-4c3c-af96-122e757b18d2"/>
     <xsd:element name="properties">
       <xsd:complexType>
         <xsd:sequence>
@@ -5065,6 +5066,11 @@
                 <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
           </xsd:element>
@@ -5090,6 +5096,43 @@
         <xsd:restriction base="dms:Note"/>
       </xsd:simpleType>
     </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="11" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="12" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="13" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="15" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Etiquetas de Imagem" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="1374c586-51ca-419d-b13a-551147e70874" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="59ec22bb-74c1-4c3c-af96-122e757b18d2" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="16" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{281605ea-d3cc-4310-8c97-aa0e64c9f496}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="59ec22bb-74c1-4c3c-af96-122e757b18d2">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
   </xsd:schema>
   <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
     <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
@@ -5100,8 +5143,8 @@
         <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de Conteúdo"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
         <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
         <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
@@ -5201,12 +5244,17 @@
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
+  <documentManagement>
+    <TaxCatchAll xmlns="59ec22bb-74c1-4c3c-af96-122e757b18d2" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="32f33a6e-f018-4796-a6d6-b8c30f0661e9">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
 </p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7855ED32-D8D5-45D4-B0B8-F2C65BAFB002}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ADBC6C95-0C98-420B-924B-89D3761F463D}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
Migração de dados do Sharepoint (#159)
Esta migração de dados pretende uniformizar o local de desenvolvimento
no GitHub.
</commit_message>
<xml_diff>
--- a/01-artefactos-de-gestao/01.01-templates/backlog-projeto-template-v05.xlsx
+++ b/01-artefactos-de-gestao/01.01-templates/backlog-projeto-template-v05.xlsx
@@ -5053,9 +5053,10 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100293B981485C9E24DAE651C97D9FBC267" ma:contentTypeVersion="3" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="81e1889baf096e0f1fabc7e628f510b3">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="32f33a6e-f018-4796-a6d6-b8c30f0661e9" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4b8b816b6954550eb9ea5c593f5cc868" ns2:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100293B981485C9E24DAE651C97D9FBC267" ma:contentTypeVersion="9" ma:contentTypeDescription="Criar um novo documento." ma:contentTypeScope="" ma:versionID="67106ac685bde41cc0caab8279921af5">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="32f33a6e-f018-4796-a6d6-b8c30f0661e9" xmlns:ns3="59ec22bb-74c1-4c3c-af96-122e757b18d2" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="6a225e97788944c998cfd0bee463245c" ns2:_="" ns3:_="">
     <xsd:import namespace="32f33a6e-f018-4796-a6d6-b8c30f0661e9"/>
+    <xsd:import namespace="59ec22bb-74c1-4c3c-af96-122e757b18d2"/>
     <xsd:element name="properties">
       <xsd:complexType>
         <xsd:sequence>
@@ -5065,6 +5066,11 @@
                 <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
           </xsd:element>
@@ -5090,6 +5096,43 @@
         <xsd:restriction base="dms:Note"/>
       </xsd:simpleType>
     </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="11" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="12" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="13" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="15" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Etiquetas de Imagem" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="1374c586-51ca-419d-b13a-551147e70874" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="59ec22bb-74c1-4c3c-af96-122e757b18d2" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="16" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{281605ea-d3cc-4310-8c97-aa0e64c9f496}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="59ec22bb-74c1-4c3c-af96-122e757b18d2">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
   </xsd:schema>
   <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
     <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
@@ -5100,8 +5143,8 @@
         <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de Conteúdo"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
         <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
         <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
@@ -5201,12 +5244,17 @@
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
+  <documentManagement>
+    <TaxCatchAll xmlns="59ec22bb-74c1-4c3c-af96-122e757b18d2" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="32f33a6e-f018-4796-a6d6-b8c30f0661e9">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
 </p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7855ED32-D8D5-45D4-B0B8-F2C65BAFB002}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ADBC6C95-0C98-420B-924B-89D3761F463D}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>